<commit_message>
test(xlsx): add cross-sheet formula references to the complex sample
Extend the styled fixture with a `Summary` sheet whose formulas reference other
sheets — `=SUM(Sales!D3:D5)`, `=Sales!D3`, and `=Sales!D6*'Meta Data'!B3` (a
sheet name with a space, so quoting is exercised). Renames Meta -> "Meta Data".

- fromXlsx preserves cross-sheet formula text verbatim (complex.spec.ts)
- engine integration: importing the workbook into one shared registry and
  giving each sheet a unique id resolves the cross-sheet formulas
  (Summary B1=17, B2=4.5, B3~=2.601) (sheet-integration.spec.ts)
- Storybook demo now renders every imported sheet in a shared book, so
  cross-sheet references re-evaluate live; e2e asserts Summary!B2 = 17
- add @types/node so the fixture-reading specs typecheck

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/storybook/stories/io/sample.xlsx
+++ b/packages/storybook/stories/io/sample.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Sales" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Meta" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Meta Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +39,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
   <fills count="5">
@@ -89,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -108,6 +113,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -633,4 +642,64 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Cross-sheet Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B2" s="4">
+        <f>SUM(Sales!D3:D5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Top Product</t>
+        </is>
+      </c>
+      <c r="B3" s="4">
+        <f>Sales!D3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Weighted</t>
+        </is>
+      </c>
+      <c r="B4" s="4">
+        <f>Sales!D6*'Meta Data'!B3</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(xlsx): import column widths and row heights
Read explicit <cols customWidth> widths and <row customHeight> heights and map
them (converted to pixels) onto the column-/row-header cells (ch(col)/rh(row)),
so imported sheets keep their sizing. Sheet-wide col spans are skipped to avoid
creating thousands of header cells.

- read.ts parses cols/rows; complex fixture varies widths/heights
- complex.spec.ts asserts the imported px sizes; e2e checks a wide vs narrow column
- README updated

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/storybook/stories/io/sample.xlsx
+++ b/packages/storybook/stories/io/sample.xlsx
@@ -485,18 +485,19 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Q3 Sales Report</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Product</t>
@@ -596,6 +597,10 @@
   </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
@@ -656,7 +661,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Cross-sheet Summary</t>

</xml_diff>